<commit_message>
Update: Add more biomes, edit scenarios
</commit_message>
<xml_diff>
--- a/tts_envs/data/tiles.xlsx
+++ b/tts_envs/data/tiles.xlsx
@@ -19,7 +19,7 @@
     <definedName name="bludgeoning">_values!$L$3:$L$4</definedName>
     <definedName name="channeling">_values!$P$3:$P$4</definedName>
     <definedName name="consumable">_values!$G$3:$G$10</definedName>
-    <definedName name="goods">_values!$H$3:$H$7</definedName>
+    <definedName name="goods">_values!$H$3:$H$8</definedName>
     <definedName name="hacking">_values!$J$3:$J$4</definedName>
     <definedName name="heavy">_values!$T$3:$T$6</definedName>
     <definedName name="infusing">_values!$R$3:$R$10</definedName>
@@ -48072,6 +48072,11 @@
           <t>rune</t>
         </is>
       </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>contraband</t>
+        </is>
+      </c>
       <c r="I8" t="inlineStr">
         <is>
           <t>2H Staff</t>
@@ -48438,6 +48443,11 @@
       </c>
     </row>
     <row r="31">
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>contraband</t>
+        </is>
+      </c>
       <c r="I31" t="inlineStr">
         <is>
           <t>meat</t>

</xml_diff>

<commit_message>
Update: Update default meeple colors
</commit_message>
<xml_diff>
--- a/tts_envs/data/tiles.xlsx
+++ b/tts_envs/data/tiles.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="items" sheetId="1" state="visible" r:id="rId1"/>
@@ -21445,7 +21445,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>item_template</t>
+          <t>skill_template</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -21530,7 +21530,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>item_template</t>
+          <t>skill_template</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -21615,7 +21615,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>item_template</t>
+          <t>skill_template</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -21700,7 +21700,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>item_template</t>
+          <t>skill_template</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -21785,7 +21785,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>item_template</t>
+          <t>skill_template</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -21870,7 +21870,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>item_template</t>
+          <t>skill_template</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -21955,7 +21955,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>item_template</t>
+          <t>skill_template</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -22040,7 +22040,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>item_template</t>
+          <t>skill_template</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -22125,7 +22125,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>item_template</t>
+          <t>skill_template</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -22210,7 +22210,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>item_template</t>
+          <t>skill_template</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -22295,7 +22295,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>item_template</t>
+          <t>skill_template</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -22380,7 +22380,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>item_template</t>
+          <t>skill_template</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -22465,7 +22465,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>item_template</t>
+          <t>skill_template</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -22550,7 +22550,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>item_template</t>
+          <t>skill_template</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -22635,7 +22635,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>item_template</t>
+          <t>skill_template</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -22720,7 +22720,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>item_template</t>
+          <t>skill_template</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -22805,7 +22805,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>item_template</t>
+          <t>skill_template</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -22890,7 +22890,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>item_template</t>
+          <t>skill_template</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -22975,7 +22975,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>item_template</t>
+          <t>skill_template</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -23060,7 +23060,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>item_template</t>
+          <t>skill_template</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -23145,7 +23145,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>item_template</t>
+          <t>skill_template</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -23230,7 +23230,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>item_template</t>
+          <t>skill_template</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -23315,7 +23315,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>item_template</t>
+          <t>skill_template</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -23400,7 +23400,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>item_template</t>
+          <t>skill_template</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -23485,7 +23485,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>item_template</t>
+          <t>skill_template</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -23570,7 +23570,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>item_template</t>
+          <t>skill_template</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -23655,7 +23655,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>item_template</t>
+          <t>skill_template</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -23740,7 +23740,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>item_template</t>
+          <t>skill_template</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -23825,7 +23825,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>item_template</t>
+          <t>skill_template</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -23910,7 +23910,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>item_template</t>
+          <t>skill_template</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -23995,7 +23995,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>item_template</t>
+          <t>skill_template</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -24080,7 +24080,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>item_template</t>
+          <t>skill_template</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -24165,7 +24165,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>item_template</t>
+          <t>skill_template</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -24250,7 +24250,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>item_template</t>
+          <t>skill_template</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -24335,7 +24335,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>item_template</t>
+          <t>skill_template</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -24420,7 +24420,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>item_template</t>
+          <t>skill_template</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -24505,7 +24505,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>item_template</t>
+          <t>skill_template</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -24590,7 +24590,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>item_template</t>
+          <t>skill_template</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -24675,7 +24675,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>item_template</t>
+          <t>skill_template</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -24760,7 +24760,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>item_template</t>
+          <t>skill_template</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -24845,7 +24845,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>item_template</t>
+          <t>skill_template</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -24930,7 +24930,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>item_template</t>
+          <t>skill_template</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -25015,7 +25015,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>item_template</t>
+          <t>skill_template</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -25100,7 +25100,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>item_template</t>
+          <t>skill_template</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -25185,7 +25185,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>item_template</t>
+          <t>skill_template</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -25270,7 +25270,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>item_template</t>
+          <t>skill_template</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -25355,7 +25355,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>item_template</t>
+          <t>skill_template</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -25440,7 +25440,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>item_template</t>
+          <t>skill_template</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">

</xml_diff>